<commit_message>
feat: mobile UI, patent sync UX, campaign delete cascade, responsive QA, AI prompt system
- Mobile: bottom tab bar (4+More), header logo only, responsive headers
- Patent sync: Toast notifications, NEW badge on synced items
- Campaign delete: RPC cascade with listing_snapshot preservation
- Reports delete: RLS policy for owner/admin
- Campaign detail: listing panel redesign with Amazon link + Create Report
- Dashboard: masonry widget improvements, AI accuracy widget stub
- AI prompts: DB-backed prompt versioning + optimizer pipeline (Phase 1-4)
- Dark mode: surface opacity fixes for visibility
- Responsive QA: full breakpoint inspection fixes
- Toast system + ScrollTabs component
- E2E test suite (responsive QA)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/01-plan/오류 수정 리스트.xlsx
+++ b/docs/01-plan/오류 수정 리스트.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hoon/Library/Mobile Documents/com~apple~CloudDocs/Documents/Claude/code/IP project /docs/01-plan/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hoon/Library/Mobile Documents/com~apple~CloudDocs/Documents/Claude Cloud/code/ip-project/docs/01-plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0CF558B-DB24-DB46-9D7B-932BE3641813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A2FD7BD-8B74-084C-9373-98AC971F2FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="700" windowWidth="29500" windowHeight="21680" xr2:uid="{FA8CC4F2-B5FE-7B45-A0C6-C44C9F831B03}"/>
+    <workbookView xWindow="48420" yWindow="-28200" windowWidth="33980" windowHeight="21640" xr2:uid="{FA8CC4F2-B5FE-7B45-A0C6-C44C9F831B03}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="오류 수정 리스트" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>날짜</t>
   </si>
@@ -195,7 +195,40 @@
     <t>크리티컬</t>
   </si>
   <si>
-    <t>Notice 오너는 신규 / 수정 / 삭제 권한, 에디터는 신규 권한 필요. 그외는 Notice 는 팝업 창이나 노티로만 받음. </t>
+    <t xml:space="preserve">신규 노티 만들려고 하면 Could not find the table 'public.notices' in the schema cache 뜨고 세이브 안됨 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">스크린샷 Screenshot 2026-03-04 at 16.45.44 보면 아마존 URL 이 amazon.com/dp/ 이렇게 시작 안해 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">캠패인에서 콜레팅 된 바이로레이션 리스팅은 리포트 큐에서 볼수 있는 연결된 리스팅이어야 한다. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">리포트 큐에서 Asin 눌르고 오른쪽 창 나오고 또 디테일 눌러야 되는데 이 액스트라 스탭 빼고 바로 디테일로 가면 좋을듯 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">어플라이 탬플릿 눌렀을때 나오는 사이트 창에 디자인완성이 안되어 있음 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">리포트 디테일에서 뒤로가기 버튼.. 아니 모든 디로가기 버튼이 좀더 잘 보이고 직관적으면 좋겠음 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">컴플릿트 리포트 에서 리스팅 들어가보면 리포트 큐로 돌아감 </t>
+  </si>
+  <si>
+    <t>오너와 관리자는 신고리포트를 삭제 할수 있는 권한 필요함 그리고 벌크단위 삭제도 필요함</t>
+  </si>
+  <si>
+    <t xml:space="preserve">벌크 단위로 서빗도 같이 필요함 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">설정에 익스텐션 페이지 디자인 필요함 지금은 너무 디자인 안된 느낌 </t>
+  </si>
+  <si>
+    <t>3.5.2026</t>
+  </si>
+  <si>
+    <t>설정에 익스텐션이름이 Download sentinel-extension-v1.0.0.zip</t>
   </si>
 </sst>
 </file>
@@ -774,7 +807,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -813,7 +846,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -839,7 +872,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -867,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -880,7 +913,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -895,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -908,7 +941,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -923,7 +956,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -936,7 +969,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -949,24 +982,32 @@
         <v>0</v>
       </c>
       <c r="E16" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="9"/>
-      <c r="C17" s="8"/>
+      <c r="C17" s="8" t="s">
+        <v>21</v>
+      </c>
       <c r="D17" s="11" t="b">
         <v>0</v>
       </c>
       <c r="E17" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="4"/>
+      <c r="A18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="5">
+        <v>5</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="D18" s="7" t="b">
         <v>0</v>
       </c>
@@ -977,7 +1018,9 @@
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="9"/>
-      <c r="C19" s="8"/>
+      <c r="C19" s="8" t="s">
+        <v>23</v>
+      </c>
       <c r="D19" s="11" t="b">
         <v>0</v>
       </c>
@@ -988,7 +1031,9 @@
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="4"/>
       <c r="B20" s="5"/>
-      <c r="C20" s="4"/>
+      <c r="C20" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="D20" s="7" t="b">
         <v>0</v>
       </c>
@@ -999,7 +1044,9 @@
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="9"/>
-      <c r="C21" s="8"/>
+      <c r="C21" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="D21" s="11" t="b">
         <v>0</v>
       </c>
@@ -1010,7 +1057,9 @@
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
       <c r="B22" s="5"/>
-      <c r="C22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="D22" s="7" t="b">
         <v>0</v>
       </c>
@@ -1021,7 +1070,9 @@
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="9"/>
-      <c r="C23" s="8"/>
+      <c r="C23" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="D23" s="11" t="b">
         <v>0</v>
       </c>
@@ -1032,7 +1083,9 @@
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
       <c r="B24" s="5"/>
-      <c r="C24" s="4"/>
+      <c r="C24" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="D24" s="7" t="b">
         <v>0</v>
       </c>
@@ -1043,7 +1096,9 @@
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="9"/>
-      <c r="C25" s="8"/>
+      <c r="C25" s="8" t="s">
+        <v>28</v>
+      </c>
       <c r="D25" s="11" t="b">
         <v>0</v>
       </c>
@@ -1054,7 +1109,9 @@
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="5"/>
-      <c r="C26" s="4"/>
+      <c r="C26" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="D26" s="7" t="b">
         <v>0</v>
       </c>

</xml_diff>